<commit_message>
Daily scrape output - 2026-08-04
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_odds_data.xlsx
+++ b/outputs/pinnacle_odds_data.xlsx
@@ -555,109 +555,85 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/universitatea-cluj-vs-botosani/1632737321</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/japs-vs-mikkelin-palloilijat/1633170564</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-03 15:30</t>
+          <t>2026-08-07 15:30</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>JaPS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Mikkelin Palloilijat</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>2.120</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>3.530</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>3.200</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>-0.25</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>1.854</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>3.580</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>4.330</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>-0.5</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>1.862</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2.000</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>9.5</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>1.826</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1.934</t>
-        </is>
-      </c>
+          <t>1.952</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2.040</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>-1.5</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>1.826</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>1.877</t>
-        </is>
-      </c>
+          <t>1.900</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
@@ -668,109 +644,85 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/sjk-vs-hjk-helsinki/1632709805</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/petrolul-ploiesti-vs-otelul-galati/1632977569</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-03 16:00</t>
+          <t>2026-08-07 15:30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SJK</t>
+          <t>Petrolul Ploiesti</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Otelul Galati</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3.370</t>
+          <t>2.800</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>4.070</t>
+          <t>2.930</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>2.750</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2.040</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>10.5</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1.980</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>1.813</t>
-        </is>
-      </c>
+          <t>1.884</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.787</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1.980</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>1.943</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>1.819</t>
-        </is>
-      </c>
+          <t>2.010</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
@@ -781,109 +733,85 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/ranheim-vs-haugesund/1632977665</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/sjk-vs-gnistan/1632871196</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-03 17:00</t>
+          <t>2026-08-07 16:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ranheim</t>
+          <t>SJK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Haugesund</t>
+          <t>Gnistan</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:26</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3.200</t>
+          <t>2.180</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>4.350</t>
+          <t>3.720</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>3.110</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>1.909</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1.943</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1.961</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
           <t>1.877</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1.980</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>1.934</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>1.826</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>1.854</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>1.990</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>+0.5</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>1.900</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>1.819</t>
-        </is>
-      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
@@ -894,109 +822,85 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/cracovia-krakow-vs-pogon-szczecin/1632854811</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/polonia-bytom-vs-pogon-siedlce/1633170573</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-03 17:00</t>
+          <t>2026-08-07 16:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cracovia Krakow</t>
+          <t>Polonia Bytom</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Pogon Szczecin</t>
+          <t>Pogon Siedlce</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2.350</t>
+          <t>1.763</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3.000</t>
+          <t>3.780</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3.580</t>
+          <t>4.180</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>1.813</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
           <t>1.909</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1.840</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>1.961</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>2.25</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>1.990</t>
-        </is>
-      </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>1.877</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>-1.0</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>1.769</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>1.952</t>
-        </is>
-      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
@@ -1007,87 +911,75 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/chrobry-glogow-vs-odra-opole/1632999616</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/ostersunds-fk-vs-sundsvall/1633170587</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-03 17:00</t>
+          <t>2026-08-07 17:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Chrobry Glogow</t>
+          <t>Ostersunds FK</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Odra Opole</t>
+          <t>Sundsvall</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:27</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2.230</t>
+          <t>1.460</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3.370</t>
+          <t>4.110</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3.280</t>
+          <t>7.020</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1.925</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>10.5</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>1.980</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>1.781</t>
-        </is>
-      </c>
+          <t>1.990</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1095,21 +987,9 @@
           <t>1.934</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>-0.5</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>1.900</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>1.813</t>
-        </is>
-      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
@@ -1120,47 +1000,47 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/orebro-sk-vs-varnamo/1632985475</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/polonia-warsaw-vs-ruch-chorzow/1633177743</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-03 17:05</t>
+          <t>2026-08-07 18:30</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>Ruch Chorzow</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2.300</t>
+          <t>2.120</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3.500</t>
+          <t>3.490</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3.050</t>
+          <t>3.250</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1170,29 +1050,17 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1.862</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>1.877</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>1.884</t>
-        </is>
-      </c>
+          <t>1.961</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>2.75</t>
@@ -1200,29 +1068,17 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1.840</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>-1.0</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>1.869</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>1.854</t>
-        </is>
-      </c>
+          <t>1.833</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
@@ -1233,109 +1089,85 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/fcsb-vs-farul-constanta/1632737323</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/operario-ferroviario-vs-sao-bernardo/1633177789</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-03 18:30</t>
+          <t>2026-08-07 22:30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Operario Ferroviario</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Farul Constanta</t>
+          <t>Sao Bernardo</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1.709</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>4.070</t>
+          <t>3.380</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.520</t>
+          <t>4.190</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1.925</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>1.909</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>1.854</t>
-        </is>
-      </c>
+          <t>1.917</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1.877</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>-2.0</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>1.806</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>1.909</t>
-        </is>
-      </c>
+          <t>2.020</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
@@ -1346,62 +1178,62 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/fc-haka-vs-jippo/1633163740</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/ceara-vs-ponte-preta/1633197947</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-07 15:00</t>
+          <t>2026-08-07 23:30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FC Haka</t>
+          <t>Ceara</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>JIPPO</t>
+          <t>Ponte Preta</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2.270</t>
+          <t>1.346</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3.520</t>
+          <t>4.770</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2.930</t>
+          <t>9.040</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-1.25</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1414,12 +1246,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
@@ -1435,62 +1267,62 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/japs-vs-mikkelin-palloilijat/1633170564</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/ljungskile-vs-oddevold/1633230235</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-07 15:30</t>
+          <t>2026-08-08 11:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>JaPS</t>
+          <t>Ljungskile</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Mikkelin Palloilijat</t>
+          <t>Oddevold</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2.130</t>
+          <t>2.550</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>3.490</t>
+          <t>3.370</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3.210</t>
+          <t>2.690</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1498,17 +1330,17 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
@@ -1524,62 +1356,62 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/petrolul-ploiesti-vs-otelul-galati/1632977569</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/radomiak-radom-vs-gornik-zabrze/1633157629</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-07 15:30</t>
+          <t>2026-08-08 12:45</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Petrolul Ploiesti</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Otelul Galati</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2.800</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2.930</t>
+          <t>3.550</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2.750</t>
+          <t>2.350</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1587,17 +1419,17 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
@@ -1613,62 +1445,62 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/polonia-bytom-vs-pogon-siedlce/1633170573</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/osters-vs-landskrona/1633242091</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-07 16:00</t>
+          <t>2026-08-08 13:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Polonia Bytom</t>
+          <t>Osters</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Pogon Siedlce</t>
+          <t>Landskrona</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1.763</t>
+          <t>2.410</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3.780</t>
+          <t>3.690</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>4.180</t>
+          <t>2.670</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1676,17 +1508,17 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
@@ -1702,47 +1534,47 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/ostersunds-fk-vs-sundsvall/1633170587</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/stal-mielec-vs-stal-rzeszow/1633247116</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-07 17:00</t>
+          <t>2026-08-08 13:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ostersunds FK</t>
+          <t>Stal Mielec</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1.444</t>
+          <t>1.595</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>4.150</t>
+          <t>4.350</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>7.270</t>
+          <t>4.610</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1752,12 +1584,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1765,7 +1597,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1791,12 +1623,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/polonia-warsaw-vs-ruch-chorzow/1633177743</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/puszcza-niepolomice-vs-odra-opole/1633248614</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-07 18:30</t>
+          <t>2026-08-08 13:30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1806,32 +1638,32 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Puszcza Niepolomice</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ruch Chorzow</t>
+          <t>Odra Opole</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2.120</t>
+          <t>2.060</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>3.490</t>
+          <t>3.480</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>3.250</t>
+          <t>3.400</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1841,12 +1673,12 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.793</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -1854,17 +1686,17 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
@@ -1880,62 +1712,62 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/uta-arad-vs-rapid-bucuresti/1632977445</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/miedz-legnica-vs-pogon-grodzisk-mazowiecki/1633248615</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-07 18:30</t>
+          <t>2026-08-08 13:30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>UTA Arad</t>
+          <t>Miedz Legnica</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Rapid Bucuresti</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2.420</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>3.140</t>
+          <t>3.870</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3.040</t>
+          <t>3.180</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2.060</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1.763</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1943,17 +1775,17 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.787</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
@@ -1969,62 +1801,62 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/operario-ferroviario-vs-sao-bernardo/1633177789</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/stabaek-vs-lyn/1633197926</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-07 22:30</t>
+          <t>2026-08-08 14:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Operario Ferroviario</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sao Bernardo</t>
+          <t>Lyn</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.425</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3.200</t>
+          <t>5.060</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>4.240</t>
+          <t>5.840</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>-1.25</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -2032,17 +1864,17 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2.040</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1.793</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
@@ -2058,62 +1890,62 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/ceara-vs-ponte-preta/1633197947</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/norrkoping-vs-brage/1633257211</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-07 23:30</t>
+          <t>2026-08-08 15:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Ceara</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Brage</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>1.346</t>
+          <t>1.549</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>4.770</t>
+          <t>4.330</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>9.040</t>
+          <t>5.160</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>-1.25</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2121,17 +1953,17 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
@@ -2147,62 +1979,62 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/falkenbergs-vs-nordic-united/1633242049</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/kapa-vs-eif/1633260738</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-08 11:00</t>
+          <t>2026-08-08 15:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>KaPa</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Nordic United</t>
+          <t>EIF</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2.140</t>
+          <t>2.790</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>3.640</t>
+          <t>3.410</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>3.120</t>
+          <t>2.420</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.769</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2215,12 +2047,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
@@ -2236,62 +2068,62 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/ljungskile-vs-oddevold/1633230235</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/sjk-akatemia-vs-pk-35/1633250556</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-08 11:00</t>
+          <t>2026-08-08 15:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>SJK Akatemia</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>PK-35</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2.560</t>
+          <t>3.950</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>3.370</t>
+          <t>3.390</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.680</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+0.5</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2299,17 +2131,17 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
@@ -2325,12 +2157,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/radomiak-radom-vs-gornik-zabrze/1633157629</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/pogon-szczecin-vs-motor-lublin/1633151820</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-08 12:45</t>
+          <t>2026-08-08 15:30</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2340,47 +2172,47 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Pogon Szczecin</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>Motor Lublin</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2.840</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3.480</t>
+          <t>3.310</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2.410</t>
+          <t>3.850</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1.769</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2.090</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2388,17 +2220,17 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
@@ -2414,62 +2246,62 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/osters-vs-landskrona/1633242091</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/farul-constanta-vs-csikszereda/1632971050</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-08 13:00</t>
+          <t>2026-08-08 15:30</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Osters</t>
+          <t>Farul Constanta</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Csikszereda</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:31</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2.440</t>
+          <t>1.520</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>3.640</t>
+          <t>4.150</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2.640</t>
+          <t>5.880</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -2477,17 +2309,17 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
@@ -2503,62 +2335,62 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/miedz-legnica-vs-pogon-grodzisk-mazowiecki/1633248615</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/jaro-vs-vps/1632932164</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-08 13:30</t>
+          <t>2026-08-08 16:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Miedz Legnica</t>
+          <t>Jaro</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>VPS</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:26</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>3.790</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>3.620</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
           <t>1.952</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>3.850</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>3.390</t>
-        </is>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>+0.5</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -2566,7 +2398,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -2576,7 +2408,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1.781</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
@@ -2592,62 +2424,62 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/stal-mielec-vs-stal-rzeszow/1633247116</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/korona-kielce-vs-legia-warsaw/1633157630</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-08 13:30</t>
+          <t>2026-08-08 18:15</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Stal Mielec</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1.595</t>
+          <t>2.820</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>4.350</t>
+          <t>3.200</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4.610</t>
+          <t>2.580</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -2655,17 +2487,17 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
@@ -2681,62 +2513,62 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/stabaek-vs-lyn/1633197926</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/dinamo-bucuresti-vs-voluntari/1632977444</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-08 14:00</t>
+          <t>2026-08-08 18:30</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Dinamo Bucuresti</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Lyn</t>
+          <t>Voluntari</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:31</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>1.450</t>
+          <t>1.518</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>4.810</t>
+          <t>4.400</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>5.810</t>
+          <t>5.430</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>-1.25</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -2744,17 +2576,17 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="S24" t="inlineStr"/>
@@ -2770,62 +2602,62 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/norrkoping-vs-brage/1633257211</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/vila-nova-vs-sport-recife/1633257267</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-08-08 15:00</t>
+          <t>2026-08-08 19:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>Vila Nova</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Sport Recife</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>1.549</t>
+          <t>2.230</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>4.350</t>
+          <t>3.040</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>5.160</t>
+          <t>3.590</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -2833,17 +2665,17 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
@@ -2859,62 +2691,62 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/kapa-vs-eif/1633260738</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/botafogo-sp-vs-america-mineiro/1633262897</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-08 15:00</t>
+          <t>2026-08-08 21:30</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>KaPa</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>EIF</t>
+          <t>America Mineiro</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2.790</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>3.410</t>
+          <t>3.170</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2.420</t>
+          <t>4.680</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>1.769</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -2922,17 +2754,17 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
@@ -2948,62 +2780,62 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/sjk-akatemia-vs-pk-35/1633250556</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/kups-vs-tps/1632932104</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-08 15:00</t>
+          <t>2026-08-09 12:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SJK Akatemia</t>
+          <t>KuPS</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PK-35</t>
+          <t>TPS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:26</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>4.000</t>
+          <t>1.462</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3.390</t>
+          <t>4.730</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>6.180</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>-1.25</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -3011,17 +2843,17 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>1.781</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
@@ -3037,62 +2869,62 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/jaro-vs-vps/1632932164</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/hjk-klubi-04-vs-ktp/1633292608</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-08 16:00</t>
+          <t>2026-08-09 12:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Jaro</t>
+          <t>HJK Klubi 04</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>VPS</t>
+          <t>KTP</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>3.680</t>
+          <t>4.500</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>3.530</t>
+          <t>4.090</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>1.649</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>+0.75</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
+          <t>1.970</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
           <t>1.833</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>2.020</t>
         </is>
       </c>
       <c r="M28" t="inlineStr"/>
@@ -3100,17 +2932,17 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="S28" t="inlineStr"/>
@@ -3126,62 +2958,62 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/korona-kielce-vs-legia-warsaw/1633157630</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/lks-lodz-vs-chrobry-glogow/1633283997</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-08-08 18:15</t>
+          <t>2026-08-09 12:30</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Legia Warsaw</t>
+          <t>Chrobry Glogow</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2.850</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>3.200</t>
+          <t>3.630</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2.560</t>
+          <t>4.000</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
@@ -3189,17 +3021,17 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
@@ -3215,62 +3047,62 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/dinamo-bucuresti-vs-voluntari/1632977444</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/varbergs-bois-vs-sandvikens-if/1633284007</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-08-08 18:30</t>
+          <t>2026-08-09 13:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Dinamo Bucuresti</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Voluntari</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>1.507</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>4.500</t>
+          <t>3.900</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>5.430</t>
+          <t>3.740</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="M30" t="inlineStr"/>
@@ -3278,17 +3110,17 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
@@ -3304,62 +3136,62 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/vila-nova-vs-sport-recife/1633257267</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/inter-turku-vs-fc-lahti/1633247173</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-08-08 19:00</t>
+          <t>2026-08-09 14:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Vila Nova</t>
+          <t>Inter Turku</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>FC Lahti</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:26</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2.260</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>3.020</t>
+          <t>3.760</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>3.550</t>
+          <t>4.280</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
@@ -3367,17 +3199,17 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
@@ -3393,62 +3225,62 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/botafogo-sp-vs-america-mineiro/1633262897</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/ac-oulu-vs-hjk-helsinki/1632926980</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-08 21:30</t>
+          <t>2026-08-09 15:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Finland - Veikkausliiga</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>AC Oulu</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>HJK Helsinki</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:26</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>3.270</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>3.170</t>
+          <t>3.410</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>4.680</t>
+          <t>2.220</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="M32" t="inlineStr"/>
@@ -3456,17 +3288,17 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
@@ -3482,12 +3314,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/kups-vs-tps/1632932104</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/ilves-vs-ifk-mariehamn/1633250529</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-08-09 12:00</t>
+          <t>2026-08-09 15:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3497,47 +3329,47 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>KuPS</t>
+          <t>Ilves</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>TPS</t>
+          <t>IFK Mariehamn</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:26</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>1.462</t>
+          <t>1.281</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>4.730</t>
+          <t>6.030</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>6.180</t>
+          <t>8.530</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>-1.25</t>
+          <t>-1.75</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="M33" t="inlineStr"/>
@@ -3545,17 +3377,17 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
@@ -3571,62 +3403,62 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/hjk-klubi-04-vs-ktp/1633292608</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/sogndal-vs-bryne/1633262887</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-09 12:00</t>
+          <t>2026-08-09 15:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>HJK Klubi 04</t>
+          <t>Sogndal</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>KTP</t>
+          <t>Bryne</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>4.730</t>
+          <t>2.540</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>4.140</t>
+          <t>3.830</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>1.613</t>
+          <t>2.450</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>+0.75</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>1.781</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="M34" t="inlineStr"/>
@@ -3634,17 +3466,17 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="S34" t="inlineStr"/>
@@ -3660,62 +3492,62 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/varbergs-bois-vs-sandvikens-if/1633284007</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/asane-fotball-vs-kongsvinger/1633265670</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-09 13:00</t>
+          <t>2026-08-09 15:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Sandvikens IF</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>5.130</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>3.870</t>
+          <t>4.960</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>3.720</t>
+          <t>1.485</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>+1.25</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
@@ -3723,17 +3555,17 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1.793</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
@@ -3749,57 +3581,57 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/inter-turku-vs-fc-lahti/1633247173</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/strommen-vs-ranheim/1633262892</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-09 14:00</t>
+          <t>2026-08-09 15:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>FC Lahti</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>2.600</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>3.800</t>
+          <t>3.820</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>4.420</t>
+          <t>2.410</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -3812,17 +3644,17 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="S36" t="inlineStr"/>
@@ -3838,62 +3670,62 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/athletic-club-vs-criciuma/1633292438</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/stromsgodset-vs-egersunds/1633262886</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-09 14:00</t>
+          <t>2026-08-09 15:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Stromsgodset</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>Egersunds</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>3.200</t>
+          <t>1.444</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2.970</t>
+          <t>5.060</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2.470</t>
+          <t>5.570</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>-1.25</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>1.769</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2.090</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="M37" t="inlineStr"/>
@@ -3901,17 +3733,17 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
@@ -3927,7 +3759,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-veikkausliiga/ilves-vs-ifk-mariehamn/1633250529</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/haugesund-vs-raufoss/1633265656</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3937,52 +3769,52 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Finland - Veikkausliiga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Ilves</t>
+          <t>Haugesund</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>IFK Mariehamn</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>1.289</t>
+          <t>1.291</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>6.050</t>
+          <t>6.010</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>8.600</t>
+          <t>7.330</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>-1.5</t>
+          <t>-1.75</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
@@ -3990,17 +3822,17 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
@@ -4041,22 +3873,22 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>3.910</t>
+          <t>3.820</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>3.900</t>
+          <t>3.640</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4066,12 +3898,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
@@ -4084,12 +3916,12 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="S39" t="inlineStr"/>
@@ -4105,62 +3937,62 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/sogndal-vs-bryne/1633262887</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/lech-poznan-vs-piast-gliwice/1633257214</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-09 15:00</t>
+          <t>2026-08-09 15:30</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Sogndal</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Bryne</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2.520</t>
+          <t>1.606</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>3.860</t>
+          <t>4.130</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2.450</t>
+          <t>5.080</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="M40" t="inlineStr"/>
@@ -4168,17 +4000,17 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
@@ -4194,62 +4026,62 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/stromsgodset-vs-egersunds/1633262886</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/universitatea-craiova-vs-arges-pitesti/1632971047</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-09 15:00</t>
+          <t>2026-08-09 15:30</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Universitatea Craiova</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Egersunds</t>
+          <t>Arges Pitesti</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:31</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>1.448</t>
+          <t>1.546</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>5.030</t>
+          <t>3.960</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>5.560</t>
+          <t>5.920</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>-1.25</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
@@ -4257,17 +4089,17 @@
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="S41" t="inlineStr"/>
@@ -4283,62 +4115,62 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/asane-fotball-vs-kongsvinger/1633265670</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/jagiellonia-bialystok-vs-widzew-lodz/1633151821</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-09 15:00</t>
+          <t>2026-08-09 18:15</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Asane Fotball</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>5.620</t>
+          <t>2.460</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>5.200</t>
+          <t>3.200</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>1.429</t>
+          <t>2.980</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>+1.25</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>2.110</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.757</t>
         </is>
       </c>
       <c r="M42" t="inlineStr"/>
@@ -4346,17 +4178,17 @@
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="S42" t="inlineStr"/>
@@ -4372,62 +4204,62 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/lech-poznan-vs-piast-gliwice/1633257214</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/gremio-novorizontino-vs-juventude/1633296951</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-08-09 15:30</t>
+          <t>2026-08-09 19:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Gremio Novorizontino</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>1.609</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>4.120</t>
+          <t>3.070</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>5.080</t>
+          <t>4.130</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2.060</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>1.793</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="M43" t="inlineStr"/>
@@ -4435,17 +4267,17 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
@@ -4461,62 +4293,62 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/universitatea-craiova-vs-arges-pitesti/1632971047</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/nautico-vs-atletico-goianiense/1633294724</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-08-09 15:30</t>
+          <t>2026-08-09 19:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Nautico</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Arges Pitesti</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:29</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>1.534</t>
+          <t>2.230</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>3.990</t>
+          <t>3.320</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>6.000</t>
+          <t>3.270</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="M44" t="inlineStr"/>
@@ -4524,17 +4356,17 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="S44" t="inlineStr"/>
@@ -4550,47 +4382,47 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/jagiellonia-bialystok-vs-widzew-lodz/1633151821</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/norrby-vs-orebro-sk/1633306165</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-08-09 18:15</t>
+          <t>2026-08-10 17:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>Norrby</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Orebro SK</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-08-03 09:33</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2.370</t>
+          <t>2.280</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>3.200</t>
+          <t>3.390</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>3.120</t>
+          <t>3.050</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4600,12 +4432,12 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="M45" t="inlineStr"/>
@@ -4613,17 +4445,17 @@
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="S45" t="inlineStr"/>
@@ -4639,62 +4471,62 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/gremio-novorizontino-vs-juventude/1633296951</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/moss-vs-odd-bk/1633304516</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-08-09 19:00</t>
+          <t>2026-08-10 17:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Gremio Novorizontino</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Odd BK</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:28</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2.070</t>
+          <t>3.020</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>3.060</t>
+          <t>4.110</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>4.050</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2.080</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>1.781</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="M46" t="inlineStr"/>
@@ -4702,12 +4534,12 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4728,52 +4560,52 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/nautico-vs-atletico-goianiense/1633294724</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/cfr-cluj-vs-universitatea-cluj/1632977568</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-08-09 19:00</t>
+          <t>2026-08-10 18:30</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Atletico Goianiense</t>
+          <t>Universitatea Cluj</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:31</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2.280</t>
+          <t>1.724</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>3.310</t>
+          <t>3.850</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>3.180</t>
+          <t>4.360</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -4783,7 +4615,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="M47" t="inlineStr"/>
@@ -4796,12 +4628,12 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="S47" t="inlineStr"/>
@@ -4817,12 +4649,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/cuiaba-vs-fortaleza/1633296987</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/goias-vs-londrina/1633332330</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-08-09 21:00</t>
+          <t>2026-08-10 22:30</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -4832,47 +4664,47 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>Goias</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Londrina</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-08-03 09:32</t>
+          <t>2026-08-04 08:30</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>1.724</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2.940</t>
+          <t>3.510</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>3.190</t>
+          <t>5.110</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2.110</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>1.757</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="M48" t="inlineStr"/>
@@ -4880,17 +4712,17 @@
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="S48" t="inlineStr"/>

</xml_diff>

<commit_message>
Daily scrape output - 2026-09-02
</commit_message>
<xml_diff>
--- a/outputs/pinnacle_odds_data.xlsx
+++ b/outputs/pinnacle_odds_data.xlsx
@@ -555,47 +555,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/helsingborgs-vs-orebro-sk/1634753632</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/rakow-czestochowa-vs-gornik-zabrze/1634917309</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-01 17:00</t>
+          <t>2026-09-03 16:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Helsingborgs</t>
+          <t>Rakow Czestochowa</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Gornik Zabrze</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2.120</t>
+          <t>2.180</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>4.000</t>
+          <t>3.480</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3.060</t>
+          <t>3.240</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -605,59 +605,35 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1.980</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>1.826</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1.934</t>
-        </is>
-      </c>
+          <t>1.952</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1.892</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>-0.5</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>1.884</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>1.826</t>
-        </is>
-      </c>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
@@ -668,109 +644,85 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/londrina-vs-juventude/1634799814</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/lech-poznan-vs-jagiellonia-bialystok/1634922656</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-01 22:30</t>
+          <t>2026-09-03 18:30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Jagiellonia Bialystok</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3.250</t>
+          <t>1.641</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3.040</t>
+          <t>4.300</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2.490</t>
+          <t>4.570</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2.110</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>10.5</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1.952</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+          <t>2.040</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1.990</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>1.847</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1.787</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>2.110</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>-0.5</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>1.877</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>1.840</t>
-        </is>
-      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
@@ -781,62 +733,62 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/rakow-czestochowa-vs-gornik-zabrze/1634917309</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/nautico-vs-botafogo-sp/1634934729</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-03 16:00</t>
+          <t>2026-09-03 23:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rakow Czestochowa</t>
+          <t>Nautico</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Gornik Zabrze</t>
+          <t>Botafogo SP</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2.180</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3.480</t>
+          <t>3.380</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3.240</t>
+          <t>3.930</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -844,17 +796,17 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
@@ -870,62 +822,62 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/lech-poznan-vs-jagiellonia-bialystok/1634922656</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/jippo-vs-ktp/1635071571</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-03 18:30</t>
+          <t>2026-09-04 15:30</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>JIPPO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Jagiellonia Bialystok</t>
+          <t>KTP</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1.609</t>
+          <t>2.650</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>4.370</t>
+          <t>3.390</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>4.730</t>
+          <t>2.550</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -933,17 +885,17 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
@@ -959,62 +911,62 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/nautico-vs-botafogo-sp/1634934729</t>
+          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/pk-35-vs-eif/1635033165</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-03 23:00</t>
+          <t>2026-09-04 16:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Finland - Ykkosliiga</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Nautico</t>
+          <t>PK-35</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Botafogo SP</t>
+          <t>EIF</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2.060</t>
+          <t>1.531</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3.260</t>
+          <t>4.270</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3.790</t>
+          <t>5.340</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.060</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1022,17 +974,17 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
+          <t>1.884</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
           <t>1.900</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>1.917</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
@@ -1048,47 +1000,47 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/jippo-vs-ktp/1635071571</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/pogon-grodzisk-mazowiecki-vs-warta-poznan/1634471572</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-04 15:30</t>
+          <t>2026-09-04 16:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>JIPPO</t>
+          <t>Pogon Grodzisk Mazowiecki</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>KTP</t>
+          <t>Warta Poznan</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.360</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3.390</t>
+          <t>3.620</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2.700</t>
+          <t>2.730</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1098,12 +1050,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.769</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>2.060</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1111,17 +1063,17 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
@@ -1137,62 +1089,62 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/finland-ykkosliiga/pk-35-vs-eif/1635033165</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/osters-vs-nordic-united/1634986672</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-04 16:00</t>
+          <t>2026-09-04 17:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Finland - Ykkosliiga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PK-35</t>
+          <t>Osters</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>EIF</t>
+          <t>Nordic United</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1.613</t>
+          <t>2.450</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>4.120</t>
+          <t>3.550</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.740</t>
+          <t>2.680</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1200,17 +1152,17 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
@@ -1226,62 +1178,62 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/pogon-grodzisk-mazowiecki-vs-warta-poznan/1634471572</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/norrkoping-vs-ljungskile/1634986676</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-04 16:00</t>
+          <t>2026-09-04 17:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Pogon Grodzisk Mazowiecki</t>
+          <t>Norrkoping</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Warta Poznan</t>
+          <t>Ljungskile</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2.360</t>
+          <t>1.483</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>3.620</t>
+          <t>4.350</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2.730</t>
+          <t>6.020</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1.769</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2.060</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1289,17 +1241,17 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
@@ -1315,62 +1267,62 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/norrkoping-vs-ljungskile/1634986676</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/cfr-cluj-vs-farul-constanta/1635033057</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-04 17:00</t>
+          <t>2026-09-04 17:30</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Norrkoping</t>
+          <t>CFR Cluj</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ljungskile</t>
+          <t>Farul Constanta</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1.515</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>4.190</t>
+          <t>3.680</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>5.810</t>
+          <t>4.040</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1378,17 +1330,17 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
@@ -1404,62 +1356,62 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/osters-vs-nordic-united/1634986672</t>
+          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/las-palmas-vs-leganes/1634992125</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-04 17:00</t>
+          <t>2026-09-04 18:30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Osters</t>
+          <t>Las Palmas</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nordic United</t>
+          <t>Leganes</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2.450</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>3.550</t>
+          <t>3.240</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2.680</t>
+          <t>4.630</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1467,17 +1419,17 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
+          <t>1.884</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
           <t>1.952</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>1.840</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
@@ -1493,62 +1445,62 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/cfr-cluj-vs-farul-constanta/1635033057</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/piast-gliwice-vs-gks-katowice/1634992126</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-04 17:30</t>
+          <t>2026-09-04 18:30</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>CFR Cluj</t>
+          <t>Piast Gliwice</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Farul Constanta</t>
+          <t>GKS Katowice</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>2.470</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3.610</t>
+          <t>3.570</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3.950</t>
+          <t>2.700</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1556,17 +1508,17 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
@@ -1582,62 +1534,62 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/las-palmas-vs-leganes/1634992125</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/nieciecza-vs-lechia-gdansk/1634471636</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30</t>
+          <t>2026-09-04 19:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Las Palmas</t>
+          <t>Nieciecza</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Leganes</t>
+          <t>Lechia Gdansk</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-01 10:55</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>1.862</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>3.960</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>3.560</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
           <t>1.869</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>3.340</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>4.590</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>-0.5</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>1.877</t>
-        </is>
-      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1645,17 +1597,17 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>2.060</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
@@ -1671,62 +1623,62 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/piast-gliwice-vs-gks-katowice/1634992126</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/criciuma-vs-cuiaba/1635033079</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30</t>
+          <t>2026-09-04 22:30</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Piast Gliwice</t>
+          <t>Criciuma</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GKS Katowice</t>
+          <t>Cuiaba</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2.470</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>3.570</t>
+          <t>3.150</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2.700</t>
+          <t>4.900</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -1734,17 +1686,17 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
@@ -1760,62 +1712,62 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/nieciecza-vs-lechia-gdansk/1634471636</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/athletic-club-vs-vila-nova/1635032991</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-04 19:00</t>
+          <t>2026-09-04 23:30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Nieciecza</t>
+          <t>Athletic Club</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lechia Gdansk</t>
+          <t>Vila Nova</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1.704</t>
+          <t>2.620</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>4.190</t>
+          <t>3.080</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4.050</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1823,17 +1775,17 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
@@ -1849,12 +1801,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/criciuma-vs-cuiaba/1635033079</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/crb-vs-america-mineiro/1635002965</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-04 22:30</t>
+          <t>2026-09-05 00:30</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1864,47 +1816,47 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Criciuma</t>
+          <t>CRB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Cuiaba</t>
+          <t>America Mineiro</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.523</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3.150</t>
+          <t>4.060</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>4.900</t>
+          <t>6.260</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -1912,17 +1864,17 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
@@ -1938,62 +1890,62 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/athletic-club-vs-vila-nova/1635032991</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/varnamo-vs-varbergs-bois/1635098680</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-04 23:30</t>
+          <t>2026-09-05 11:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Athletic Club</t>
+          <t>Varnamo</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Vila Nova</t>
+          <t>Varbergs BoIS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2.670</t>
+          <t>2.310</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>3.080</t>
+          <t>3.450</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2.820</t>
+          <t>2.950</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.806</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2001,7 +1953,7 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2011,7 +1963,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
@@ -2027,62 +1979,62 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/crb-vs-america-mineiro/1635002965</t>
+          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/real-sociedad-ii-vs-tenerife/1635103285</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-05 00:30</t>
+          <t>2026-09-05 12:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CRB</t>
+          <t>Real Sociedad II</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>America Mineiro</t>
+          <t>Tenerife</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>1.523</t>
+          <t>2.660</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>4.060</t>
+          <t>3.130</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>6.260</t>
+          <t>2.830</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2090,17 +2042,17 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
@@ -2116,47 +2068,47 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/varnamo-vs-varbergs-bois/1635098680</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/botosani-vs-sepsi/1635103286</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-05 11:00</t>
+          <t>2026-09-05 12:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Varnamo</t>
+          <t>Botosani</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Varbergs BoIS</t>
+          <t>Sepsi</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2.310</t>
+          <t>2.250</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>3.450</t>
+          <t>3.280</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.950</t>
+          <t>3.190</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2166,12 +2118,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2179,17 +2131,17 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.787</t>
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
@@ -2205,62 +2157,62 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/botosani-vs-sepsi/1635103286</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/widzew-lodz-vs-radomiak-radom/1635101521</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-05 12:00</t>
+          <t>2026-09-05 12:45</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Botosani</t>
+          <t>Widzew Lodz</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sepsi</t>
+          <t>Radomiak Radom</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2.250</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3.280</t>
+          <t>3.960</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>3.190</t>
+          <t>4.120</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2268,17 +2220,17 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
@@ -2294,57 +2246,57 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/widzew-lodz-vs-radomiak-radom/1635101521</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/oddevold-vs-falkenbergs/1635101542</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-05 12:45</t>
+          <t>2026-09-05 13:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Widzew Lodz</t>
+          <t>Oddevold</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Radomiak Radom</t>
+          <t>Falkenbergs</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>2.270</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>3.960</t>
+          <t>3.490</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>4.120</t>
+          <t>2.980</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2362,12 +2314,12 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
@@ -2408,37 +2360,37 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2.980</t>
+          <t>2.730</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>3.520</t>
+          <t>3.490</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2.250</t>
+          <t>2.450</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -2451,12 +2403,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
@@ -2472,62 +2424,62 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/oddevold-vs-falkenbergs/1635101542</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/stal-rzeszow-vs-polonia-warsaw/1634582008</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-05 13:00</t>
+          <t>2026-09-05 13:30</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Oddevold</t>
+          <t>Stal Rzeszow</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Polonia Warsaw</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2.200</t>
+          <t>3.310</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>3.510</t>
+          <t>3.670</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>3.070</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -2535,17 +2487,17 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
@@ -2586,7 +2538,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2675,7 +2627,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2739,52 +2691,52 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/stal-rzeszow-vs-polonia-warsaw/1634582008</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/asane-fotball-vs-hodd/1635113794</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-05 13:30</t>
+          <t>2026-09-05 14:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Stal Rzeszow</t>
+          <t>Asane Fotball</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Polonia Warsaw</t>
+          <t>Hodd</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>3.320</t>
+          <t>2.390</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>3.680</t>
+          <t>3.610</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>2.710</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2807,12 +2759,12 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
@@ -2828,7 +2780,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/sandnes-ulf-vs-ranheim/1635113786</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/kongsvinger-vs-raufoss/1635113904</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2843,47 +2795,47 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sandnes Ulf</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ranheim</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2.360</t>
+          <t>1.215</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3.900</t>
+          <t>6.310</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2.620</t>
+          <t>10.640</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-2.0</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>1.806</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -2891,17 +2843,17 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
@@ -2917,7 +2869,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/odd-bk-vs-stromsgodset/1635113903</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/sandnes-ulf-vs-ranheim/1635113786</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2932,47 +2884,47 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Odd BK</t>
+          <t>Sandnes Ulf</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Stromsgodset</t>
+          <t>Ranheim</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>3.300</t>
+          <t>2.310</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>4.170</t>
+          <t>3.900</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>2.680</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="M28" t="inlineStr"/>
@@ -2985,12 +2937,12 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="S28" t="inlineStr"/>
@@ -3031,22 +2983,22 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>1.367</t>
+          <t>1.332</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>5.670</t>
+          <t>5.900</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>6.170</t>
+          <t>6.640</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -3056,12 +3008,12 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
@@ -3074,12 +3026,12 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="S29" t="inlineStr"/>
@@ -3120,22 +3072,22 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>3.210</t>
+          <t>3.190</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>3.690</t>
+          <t>3.640</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2.070</t>
+          <t>2.110</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -3145,12 +3097,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="M30" t="inlineStr"/>
@@ -3163,12 +3115,12 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
@@ -3184,62 +3136,62 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/kongsvinger-vs-raufoss/1635113904</t>
+          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/sporting-gijon-vs-girona/1635113901</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-05 14:00</t>
+          <t>2026-09-05 14:15</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>Sporting Gijon</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>1.215</t>
+          <t>2.910</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>6.310</t>
+          <t>3.210</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>10.640</t>
+          <t>2.530</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>-2.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>2.070</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.793</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
@@ -3247,17 +3199,17 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
@@ -3273,62 +3225,62 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/asane-fotball-vs-hodd/1635113794</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/uta-arad-vs-csikszereda/1635119266</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-05 14:00</t>
+          <t>2026-09-05 14:30</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Asane Fotball</t>
+          <t>UTA Arad</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hodd</t>
+          <t>Csikszereda</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2.390</t>
+          <t>1.591</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>3.610</t>
+          <t>3.900</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2.710</t>
+          <t>5.410</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.75</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>1.787</t>
+          <t>1.769</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="M32" t="inlineStr"/>
@@ -3336,17 +3288,17 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
@@ -3362,62 +3314,62 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/sporting-gijon-vs-girona/1635113901</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/helsingborgs-vs-sandvikens-if/1635119281</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-05 14:15</t>
+          <t>2026-09-05 15:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Sporting Gijon</t>
+          <t>Helsingborgs</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Sandvikens IF</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2.910</t>
+          <t>2.200</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>3.210</t>
+          <t>3.920</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2.530</t>
+          <t>2.820</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2.070</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>1.793</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="M33" t="inlineStr"/>
@@ -3425,17 +3377,17 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
@@ -3451,47 +3403,47 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/uta-arad-vs-csikszereda/1635119266</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/brage-vs-sundsvall/1635113828</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-05 14:30</t>
+          <t>2026-09-05 15:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>UTA Arad</t>
+          <t>Brage</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Csikszereda</t>
+          <t>Sundsvall</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>1.606</t>
+          <t>1.689</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>3.880</t>
+          <t>3.950</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>5.350</t>
+          <t>4.480</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3501,12 +3453,12 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>1.781</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2.040</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="M34" t="inlineStr"/>
@@ -3514,17 +3466,17 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>1.925</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1.862</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="S34" t="inlineStr"/>
@@ -3540,62 +3492,62 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/brage-vs-sundsvall/1635113828</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/korona-kielce-vs-wisla-krakow/1635126642</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-05 15:00</t>
+          <t>2026-09-05 15:30</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Sweden - Superettan</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Brage</t>
+          <t>Korona Kielce</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Sundsvall</t>
+          <t>Wisla Krakow</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>1.689</t>
+          <t>2.250</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>3.950</t>
+          <t>3.570</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>4.480</t>
+          <t>3.020</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>1.892</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
@@ -3608,7 +3560,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3629,62 +3581,62 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/korona-kielce-vs-wisla-krakow/1635126642</t>
+          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/real-valladolid-vs-fc-andorra/1635126669</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-09-05 15:30</t>
+          <t>2026-09-05 16:30</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Korona Kielce</t>
+          <t>Real Valladolid</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Wisla Krakow</t>
+          <t>FC Andorra</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2.240</t>
+          <t>2.540</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>3.570</t>
+          <t>3.250</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>3.040</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="M36" t="inlineStr"/>
@@ -3692,17 +3644,17 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="S36" t="inlineStr"/>
@@ -3743,7 +3695,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3807,62 +3759,62 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/real-valladolid-vs-fc-andorra/1635126669</t>
+          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/stabaek-vs-moss/1635127055</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-09-05 16:30</t>
+          <t>2026-09-05 18:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Norway - 1st Division</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Real Valladolid</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Moss</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2.530</t>
+          <t>1.347</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>3.280</t>
+          <t>5.760</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2.860</t>
+          <t>6.440</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-1.5</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
@@ -3870,7 +3822,7 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -3880,7 +3832,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.800</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
@@ -3896,62 +3848,62 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/dinamo-bucuresti-vs-fcsb/1635126688</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/motor-lublin-vs-legia-warsaw/1635127066</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-09-05 17:30</t>
+          <t>2026-09-05 18:15</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - Ekstraklasa</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Dinamo Bucuresti</t>
+          <t>Motor Lublin</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FCSB</t>
+          <t>Legia Warsaw</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2.380</t>
+          <t>3.900</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>3.320</t>
+          <t>3.710</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2.950</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>+0.5</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>1.952</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
@@ -3959,17 +3911,17 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="S39" t="inlineStr"/>
@@ -3985,62 +3937,62 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/norway-1st-division/stabaek-vs-moss/1635127055</t>
+          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/eldense-vs-mallorca/1635127081</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-09-05 18:00</t>
+          <t>2026-09-05 19:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Norway - 1st Division</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Eldense</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Moss</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>1.347</t>
+          <t>3.550</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>5.760</t>
+          <t>3.360</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>6.440</t>
+          <t>2.120</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>-1.5</t>
+          <t>+0.25</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>2.030</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="M40" t="inlineStr"/>
@@ -4048,17 +4000,17 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
@@ -4074,62 +4026,62 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-ekstraklasa/motor-lublin-vs-legia-warsaw/1635127066</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/goias-vs-fortaleza/1635127083</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-09-05 18:15</t>
+          <t>2026-09-05 19:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Poland - Ekstraklasa</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Motor Lublin</t>
+          <t>Goias</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Legia Warsaw</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>3.900</t>
+          <t>2.550</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>3.710</t>
+          <t>2.950</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>3.100</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.740</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>2.130</t>
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
@@ -4137,17 +4089,17 @@
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>2.020</t>
         </is>
       </c>
       <c r="S41" t="inlineStr"/>
@@ -4163,7 +4115,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/eldense-vs-mallorca/1635127081</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/gremio-novorizontino-vs-avai/1635127082</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4173,52 +4125,52 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Eldense</t>
+          <t>Gremio Novorizontino</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>Avai</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>3.530</t>
+          <t>1.471</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>3.410</t>
+          <t>4.070</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2.110</t>
+          <t>7.270</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2.040</t>
+          <t>1.840</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="M42" t="inlineStr"/>
@@ -4231,7 +4183,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>2.030</t>
+          <t>2.010</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4252,12 +4204,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/gremio-novorizontino-vs-avai/1635127082</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/juventude-vs-atletico-goianiense/1635132183</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-09-05 19:00</t>
+          <t>2026-09-05 21:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4267,37 +4219,37 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Gremio Novorizontino</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Avai</t>
+          <t>Atletico Goianiense</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>1.471</t>
+          <t>2.180</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>4.070</t>
+          <t>2.960</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>7.270</t>
+          <t>3.850</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -4315,17 +4267,17 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1.819</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
@@ -4341,12 +4293,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/goias-vs-fortaleza/1635127083</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/ceara-vs-sport-recife/1635132190</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-09-05 19:00</t>
+          <t>2026-09-05 21:30</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -4356,47 +4308,47 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Goias</t>
+          <t>Ceara</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Sport Recife</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2.560</t>
+          <t>2.260</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>2.950</t>
+          <t>3.170</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>3.080</t>
+          <t>3.370</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>1.751</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2.120</t>
+          <t>1.900</t>
         </is>
       </c>
       <c r="M44" t="inlineStr"/>
@@ -4404,17 +4356,17 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>1.813</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="S44" t="inlineStr"/>
@@ -4430,62 +4382,62 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/ceara-vs-sport-recife/1635132190</t>
+          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/eibar-vs-granada/1635196862</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-09-05 21:30</t>
+          <t>2026-09-06 12:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Brazil - Serie B</t>
+          <t>Spain - Segunda</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Ceara</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Sport Recife</t>
+          <t>Granada</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2.260</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>3.170</t>
+          <t>3.480</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>3.370</t>
+          <t>3.950</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.884</t>
         </is>
       </c>
       <c r="M45" t="inlineStr"/>
@@ -4498,12 +4450,12 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="S45" t="inlineStr"/>
@@ -4519,7 +4471,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/spain-segunda-division/eibar-vs-granada/1635196862</t>
+          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/petrolul-ploiesti-vs-corvinul-hunedoara/1635196860</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -4529,42 +4481,42 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Spain - Segunda</t>
+          <t>Romania - Liga 1</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Eibar</t>
+          <t>Petrolul Ploiesti</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Granada</t>
+          <t>Corvinul Hunedoara</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:24</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>1.943</t>
+          <t>2.690</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>3.540</t>
+          <t>3.340</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>3.920</t>
+          <t>2.560</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -4574,7 +4526,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>1.900</t>
+          <t>1.847</t>
         </is>
       </c>
       <c r="M46" t="inlineStr"/>
@@ -4587,12 +4539,12 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.826</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="S46" t="inlineStr"/>
@@ -4608,62 +4560,62 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/petrolul-ploiesti-vs-corvinul-hunedoara/1635196860</t>
+          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/arka-gdynia-vs-lks-lodz/1634648982</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-09-06 12:00</t>
+          <t>2026-09-06 12:30</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Poland - 1st Liga</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Petrolul Ploiesti</t>
+          <t>Arka Gdynia</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Corvinul Hunedoara</t>
+          <t>LKS Lodz</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2.610</t>
+          <t>2.360</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>3.340</t>
+          <t>3.400</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2.640</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.769</t>
         </is>
       </c>
       <c r="M47" t="inlineStr"/>
@@ -4671,17 +4623,17 @@
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>1.826</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.869</t>
         </is>
       </c>
       <c r="S47" t="inlineStr"/>
@@ -4697,47 +4649,47 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/poland-1st-liga/arka-gdynia-vs-lks-lodz/1634648982</t>
+          <t>https://www.pinnacle.com/en/soccer/brazil-serie-b/londrina-vs-operario-ferroviario/1635193866</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-09-06 12:30</t>
+          <t>2026-09-06 14:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Poland - 1st Liga</t>
+          <t>Brazil - Serie B</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Arka Gdynia</t>
+          <t>Londrina</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>Operario Ferroviario</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2.360</t>
+          <t>2.230</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>3.400</t>
+          <t>3.310</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2.870</t>
+          <t>3.270</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -4747,12 +4699,12 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>2.050</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>1.769</t>
+          <t>1.909</t>
         </is>
       </c>
       <c r="M48" t="inlineStr"/>
@@ -4760,17 +4712,17 @@
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>1.917</t>
+          <t>1.854</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.970</t>
         </is>
       </c>
       <c r="S48" t="inlineStr"/>
@@ -4811,7 +4763,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4900,7 +4852,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4989,7 +4941,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5078,7 +5030,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -5167,22 +5119,22 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>1.292</t>
+          <t>1.298</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>5.160</t>
+          <t>5.110</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>9.260</t>
+          <t>9.090</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -5192,12 +5144,12 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.813</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="M53" t="inlineStr"/>
@@ -5256,7 +5208,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -5345,7 +5297,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5434,7 +5386,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:24</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -5523,22 +5475,22 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>1.500</t>
+          <t>1.510</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>4.390</t>
+          <t>4.360</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>6.160</t>
+          <t>6.060</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -5548,12 +5500,12 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="M57" t="inlineStr"/>
@@ -5566,12 +5518,12 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>1.970</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>1.869</t>
+          <t>1.862</t>
         </is>
       </c>
       <c r="S57" t="inlineStr"/>
@@ -5612,37 +5564,37 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>11.680</t>
+          <t>5.900</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>6.010</t>
+          <t>3.970</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>1.130</t>
+          <t>1.462</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>+2.0</t>
+          <t>+1.0</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>1.740</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.793</t>
         </is>
       </c>
       <c r="M58" t="inlineStr"/>
@@ -5655,12 +5607,12 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>1.769</t>
+          <t>1.961</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.763</t>
         </is>
       </c>
       <c r="S58" t="inlineStr"/>
@@ -5701,22 +5653,22 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:24</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2.810</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>3.340</t>
+          <t>3.190</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2.450</t>
+          <t>2.500</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -5731,7 +5683,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>1.775</t>
+          <t>1.781</t>
         </is>
       </c>
       <c r="M59" t="inlineStr"/>
@@ -5739,17 +5691,17 @@
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>1.840</t>
+          <t>1.793</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>2.000</t>
         </is>
       </c>
       <c r="S59" t="inlineStr"/>
@@ -5790,22 +5742,22 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:22</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>3.660</t>
+          <t>3.730</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>3.390</t>
+          <t>3.590</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -5815,12 +5767,12 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.925</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.877</t>
         </is>
       </c>
       <c r="M60" t="inlineStr"/>
@@ -5833,12 +5785,12 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="S60" t="inlineStr"/>
@@ -5879,22 +5831,22 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-09-01 10:57</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>1.877</t>
+          <t>1.934</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>3.710</t>
+          <t>3.650</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>3.920</t>
+          <t>3.750</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -5904,12 +5856,12 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>1.884</t>
+          <t>1.943</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>1.952</t>
+          <t>1.892</t>
         </is>
       </c>
       <c r="M61" t="inlineStr"/>
@@ -5922,12 +5874,12 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>1.980</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>1.833</t>
         </is>
       </c>
       <c r="S61" t="inlineStr"/>
@@ -5968,7 +5920,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -6032,62 +5984,62 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://www.pinnacle.com/en/soccer/romania-liga-1/universitatea-craiova-vs-universitatea-cluj/1635255961</t>
+          <t>https://www.pinnacle.com/en/soccer/sweden-superettan/orebro-sk-vs-ostersunds-fk/1635255655</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-09-07 17:30</t>
+          <t>2026-09-07 17:05</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Romania - Liga 1</t>
+          <t>Sweden - Superettan</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Universitatea Craiova</t>
+          <t>Orebro SK</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Universitatea Cluj</t>
+          <t>Ostersunds FK</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>1.653</t>
+          <t>2.760</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>4.120</t>
+          <t>3.520</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>4.510</t>
+          <t>2.390</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>-0.75</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>1.847</t>
+          <t>2.050</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>1.961</t>
+          <t>1.775</t>
         </is>
       </c>
       <c r="M63" t="inlineStr"/>
@@ -6095,17 +6047,17 @@
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>1.854</t>
+          <t>1.819</t>
         </is>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>1.934</t>
+          <t>1.980</t>
         </is>
       </c>
       <c r="S63" t="inlineStr"/>
@@ -6146,7 +6098,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-09-01 10:56</t>
+          <t>2026-09-02 10:21</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -6235,7 +6187,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-09-01 10:58</t>
+          <t>2026-09-02 10:23</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">

</xml_diff>